<commit_message>
Updated start year capacities to use the latest 860 with data for 2024 for plant and battery capacity
</commit_message>
<xml_diff>
--- a/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
+++ b/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\GBSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\GBSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68C85CB-F764-4BED-BCAC-5B594C512666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F54FC92-3C53-4C4D-9D96-341C82DD405A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1268,20 +1268,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1289,9 +1277,6 @@
     </xf>
     <xf numFmtId="167" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1302,8 +1287,23 @@
     <xf numFmtId="167" fontId="22" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="74">
@@ -1683,23 +1683,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" customWidth="1"/>
-    <col min="2" max="2" width="60.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1707,84 +1707,84 @@
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>149</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>1000</v>
       </c>
@@ -1801,14 +1801,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AK114"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.08984375" customWidth="1"/>
-    <col min="2" max="2" width="45.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" customWidth="1"/>
     <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="9" t="s">
         <v>123</v>
       </c>
@@ -1915,8 +1915,8 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1927,7 +1927,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1951,7 +1951,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
@@ -1962,7 +1962,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1970,12 +1970,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>9</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="10" t="s">
         <v>10</v>
       </c>
@@ -2195,18 +2195,18 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>13</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>-1.4527999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>-1.2109E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>2.2502999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>19</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>8.456E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>-5.6340000000000001E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>25</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>0.123014</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>27</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>5.8900000000000003E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>2.3185000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>31</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>34</v>
       </c>
@@ -3449,12 +3449,12 @@
         <v>1.1344E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>37</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>-3.3660000000000001E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>39</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>41</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>-9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>42</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>-9.68E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>43</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>6.6000000000000005E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>44</v>
       </c>
@@ -4132,12 +4132,12 @@
         <v>-4.06E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>46</v>
       </c>
@@ -4250,7 +4250,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>47</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>48</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>49</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>50</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>52</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>53</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>54</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>55</v>
       </c>
@@ -5154,7 +5154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>56</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>58</v>
       </c>
@@ -5380,12 +5380,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>60</v>
       </c>
@@ -5498,7 +5498,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>61</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>62</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>63</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>64</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>65</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>66</v>
       </c>
@@ -6176,7 +6176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>67</v>
       </c>
@@ -6289,7 +6289,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>68</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>69</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>70</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>71</v>
       </c>
@@ -6741,12 +6741,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="12" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>73</v>
       </c>
@@ -6859,7 +6859,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>74</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>75</v>
       </c>
@@ -7085,7 +7085,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>76</v>
       </c>
@@ -7198,7 +7198,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>77</v>
       </c>
@@ -7311,7 +7311,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>78</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>79</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>80</v>
       </c>
@@ -7650,7 +7650,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>81</v>
       </c>
@@ -7763,7 +7763,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>82</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>83</v>
       </c>
@@ -7989,12 +7989,12 @@
         <v>1.1053E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>86</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>-9.3640000000000008E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>87</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>-2.039E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>89</v>
       </c>
@@ -8333,7 +8333,7 @@
         <v>2.5253000000000001E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>91</v>
       </c>
@@ -8446,7 +8446,7 @@
         <v>-7.0799999999999997E-4</v>
       </c>
     </row>
-    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>93</v>
       </c>
@@ -8559,7 +8559,7 @@
         <v>6.0502E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>94</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>4.0169999999999997E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>96</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>4.7788999999999998E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>97</v>
       </c>
@@ -8898,178 +8898,178 @@
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B87" s="26" t="s">
+    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="C87" s="26"/>
-      <c r="D87" s="26"/>
-      <c r="E87" s="26"/>
-      <c r="F87" s="26"/>
-      <c r="G87" s="26"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="26"/>
-      <c r="J87" s="26"/>
-      <c r="K87" s="26"/>
-      <c r="L87" s="26"/>
-      <c r="M87" s="26"/>
-      <c r="N87" s="26"/>
-      <c r="O87" s="26"/>
-      <c r="P87" s="26"/>
-      <c r="Q87" s="26"/>
-      <c r="R87" s="26"/>
-      <c r="S87" s="26"/>
-      <c r="T87" s="26"/>
-      <c r="U87" s="26"/>
-      <c r="V87" s="26"/>
-      <c r="W87" s="26"/>
-      <c r="X87" s="26"/>
-      <c r="Y87" s="26"/>
-      <c r="Z87" s="26"/>
-      <c r="AA87" s="26"/>
-      <c r="AB87" s="26"/>
-      <c r="AC87" s="26"/>
-      <c r="AD87" s="26"/>
-      <c r="AE87" s="26"/>
-      <c r="AF87" s="26"/>
-      <c r="AG87" s="26"/>
-      <c r="AH87" s="26"/>
-      <c r="AI87" s="26"/>
-      <c r="AJ87" s="26"/>
-      <c r="AK87" s="26"/>
-    </row>
-    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C87" s="33"/>
+      <c r="D87" s="33"/>
+      <c r="E87" s="33"/>
+      <c r="F87" s="33"/>
+      <c r="G87" s="33"/>
+      <c r="H87" s="33"/>
+      <c r="I87" s="33"/>
+      <c r="J87" s="33"/>
+      <c r="K87" s="33"/>
+      <c r="L87" s="33"/>
+      <c r="M87" s="33"/>
+      <c r="N87" s="33"/>
+      <c r="O87" s="33"/>
+      <c r="P87" s="33"/>
+      <c r="Q87" s="33"/>
+      <c r="R87" s="33"/>
+      <c r="S87" s="33"/>
+      <c r="T87" s="33"/>
+      <c r="U87" s="33"/>
+      <c r="V87" s="33"/>
+      <c r="W87" s="33"/>
+      <c r="X87" s="33"/>
+      <c r="Y87" s="33"/>
+      <c r="Z87" s="33"/>
+      <c r="AA87" s="33"/>
+      <c r="AB87" s="33"/>
+      <c r="AC87" s="33"/>
+      <c r="AD87" s="33"/>
+      <c r="AE87" s="33"/>
+      <c r="AF87" s="33"/>
+      <c r="AG87" s="33"/>
+      <c r="AH87" s="33"/>
+      <c r="AI87" s="33"/>
+      <c r="AJ87" s="33"/>
+      <c r="AK87" s="33"/>
+    </row>
+    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="7" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="7" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="7" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="7" t="s">
         <v>138</v>
       </c>
@@ -9085,56 +9085,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46C8A405-A765-4E2E-A98F-140D5DD3A510}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.1796875" style="28"/>
+    <col min="1" max="1" width="17.140625" style="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="26" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="31"/>
-    </row>
-    <row r="3" spans="1:5" ht="26.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="29" t="s">
+      <c r="E2" s="38"/>
+    </row>
+    <row r="3" spans="1:5" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="29" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
         <v>160</v>
       </c>
@@ -9143,194 +9143,194 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="30">
         <v>2014</v>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="31">
         <v>155.1</v>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="32">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="D5" s="36">
+      <c r="D5" s="31">
         <v>22477.9</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="30">
         <v>2015</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="31">
         <v>206.8</v>
       </c>
-      <c r="C6" s="37">
+      <c r="C6" s="32">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="D6" s="36">
+      <c r="D6" s="31">
         <v>22568.9</v>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="30">
         <v>2016</v>
       </c>
-      <c r="B7" s="36">
+      <c r="B7" s="31">
         <v>423</v>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="32">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="31">
         <v>22752.7</v>
       </c>
-      <c r="E7" s="37">
+      <c r="E7" s="32">
         <v>0.112</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="30">
         <v>2017</v>
       </c>
-      <c r="B8" s="36">
+      <c r="B8" s="31">
         <v>632.79999999999995</v>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="32">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="D8" s="36">
+      <c r="D8" s="31">
         <v>22791.7</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="32">
         <v>0.114</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="30">
         <v>2018</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B9" s="31">
         <v>713.6</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="32">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="31">
         <v>22815.4</v>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="32">
         <v>0.108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="30">
         <v>2019</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="31">
         <v>949.8</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="32">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="31">
         <v>22754.7</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="32">
         <v>0.104</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="30">
         <v>2020</v>
       </c>
-      <c r="B11" s="36">
+      <c r="B11" s="31">
         <v>1210.3</v>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="32">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="31">
         <v>22939.599999999999</v>
       </c>
-      <c r="E11" s="37">
+      <c r="E11" s="32">
         <v>0.105</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="30">
         <v>2021</v>
       </c>
-      <c r="B12" s="36">
+      <c r="B12" s="31">
         <v>2627.6</v>
       </c>
-      <c r="C12" s="37">
+      <c r="C12" s="32">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="31">
         <v>23007.7</v>
       </c>
-      <c r="E12" s="37">
+      <c r="E12" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="30">
         <v>2022</v>
       </c>
-      <c r="B13" s="36">
+      <c r="B13" s="31">
         <v>6566.1</v>
       </c>
-      <c r="C13" s="37">
+      <c r="C13" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="31">
         <v>23033.9</v>
       </c>
-      <c r="E13" s="37">
+      <c r="E13" s="32">
         <v>0.111</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="30">
         <v>2023</v>
       </c>
-      <c r="B14" s="36">
+      <c r="B14" s="31">
         <v>11225.7</v>
       </c>
-      <c r="C14" s="37">
+      <c r="C14" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="31">
         <v>23132.1</v>
       </c>
-      <c r="E14" s="37">
+      <c r="E14" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="30">
         <v>2024</v>
       </c>
-      <c r="B15" s="36">
+      <c r="B15" s="31">
         <v>19945.099999999999</v>
       </c>
-      <c r="C15" s="37">
+      <c r="C15" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="31">
         <v>23178.5</v>
       </c>
-      <c r="E15" s="37">
+      <c r="E15" s="32">
         <v>0.114</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
         <v>161</v>
       </c>
@@ -9339,211 +9339,211 @@
       <c r="D16" s="34"/>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="35" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="36">
+      <c r="B17" s="31">
         <v>4926.3999999999996</v>
       </c>
-      <c r="C17" s="37">
+      <c r="C17" s="32">
         <v>5.5E-2</v>
       </c>
-      <c r="D17" s="36">
+      <c r="D17" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E17" s="37">
+      <c r="E17" s="32">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="35" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="36">
+      <c r="B18" s="31">
         <v>4996.7</v>
       </c>
-      <c r="C18" s="37">
+      <c r="C18" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="32">
         <v>8.8999999999999996E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="35" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B19" s="36">
+      <c r="B19" s="31">
         <v>5069.2</v>
       </c>
-      <c r="C19" s="37">
+      <c r="C19" s="32">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="D19" s="36">
+      <c r="D19" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E19" s="37">
+      <c r="E19" s="32">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="35" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="36">
+      <c r="B20" s="31">
         <v>5316.2</v>
       </c>
-      <c r="C20" s="37">
+      <c r="C20" s="32">
         <v>0.06</v>
       </c>
-      <c r="D20" s="36">
+      <c r="D20" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E20" s="37">
+      <c r="E20" s="32">
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="35" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B21" s="36">
+      <c r="B21" s="31">
         <v>6055.5</v>
       </c>
-      <c r="C21" s="37">
+      <c r="C21" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D21" s="36">
+      <c r="D21" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E21" s="37">
+      <c r="E21" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="35" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="31">
         <v>6064.5</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="32">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="D22" s="36">
+      <c r="D22" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E22" s="37">
+      <c r="E22" s="32">
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="35" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="36">
+      <c r="B23" s="31">
         <v>6555.2</v>
       </c>
-      <c r="C23" s="37">
+      <c r="C23" s="32">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E23" s="37">
+      <c r="E23" s="32">
         <v>0.159</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="35" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B24" s="36">
+      <c r="B24" s="31">
         <v>6941.6</v>
       </c>
-      <c r="C24" s="37">
+      <c r="C24" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D24" s="36">
+      <c r="D24" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E24" s="37">
+      <c r="E24" s="32">
         <v>0.16400000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="35" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B25" s="36">
+      <c r="B25" s="31">
         <v>7469.9</v>
       </c>
-      <c r="C25" s="37">
+      <c r="C25" s="32">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D25" s="36">
+      <c r="D25" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E25" s="37">
+      <c r="E25" s="32">
         <v>0.13200000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="35" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B26" s="36">
+      <c r="B26" s="31">
         <v>7958.4</v>
       </c>
-      <c r="C26" s="37">
+      <c r="C26" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D26" s="36">
+      <c r="D26" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E26" s="37">
+      <c r="E26" s="32">
         <v>8.4000000000000005E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="35" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B27" s="36">
+      <c r="B27" s="31">
         <v>8630.7000000000007</v>
       </c>
-      <c r="C27" s="37">
+      <c r="C27" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D27" s="36">
+      <c r="D27" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E27" s="37">
+      <c r="E27" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="35" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="31">
         <v>8696.4</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C28" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="32">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="34" t="s">
         <v>174</v>
       </c>
@@ -9552,211 +9552,211 @@
       <c r="D29" s="34"/>
       <c r="E29" s="34"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="35" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="31">
         <v>9168.7000000000007</v>
       </c>
-      <c r="C30" s="37">
+      <c r="C30" s="32">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D30" s="36">
+      <c r="D30" s="31">
         <v>23057.8</v>
       </c>
-      <c r="E30" s="37">
+      <c r="E30" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="35" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B31" s="36">
+      <c r="B31" s="31">
         <v>9236.4</v>
       </c>
-      <c r="C31" s="37">
+      <c r="C31" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D31" s="36">
+      <c r="D31" s="31">
         <v>23057.8</v>
       </c>
-      <c r="E31" s="37">
+      <c r="E31" s="32">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="35" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B32" s="36">
+      <c r="B32" s="31">
         <v>9318.4</v>
       </c>
-      <c r="C32" s="37">
+      <c r="C32" s="32">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D32" s="36">
+      <c r="D32" s="31">
         <v>23137.8</v>
       </c>
-      <c r="E32" s="37">
+      <c r="E32" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="35" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="31">
         <v>9621.5</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="32">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E33" s="37">
+      <c r="E33" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="35" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B34" s="36">
+      <c r="B34" s="31">
         <v>9791.5</v>
       </c>
-      <c r="C34" s="37">
+      <c r="C34" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D34" s="36">
+      <c r="D34" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E34" s="37">
+      <c r="E34" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="35" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B35" s="36">
+      <c r="B35" s="31">
         <v>9943.1</v>
       </c>
-      <c r="C35" s="37">
+      <c r="C35" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D35" s="36">
+      <c r="D35" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E35" s="37">
+      <c r="E35" s="32">
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="35" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="31">
         <v>10846.6</v>
       </c>
-      <c r="C36" s="37">
+      <c r="C36" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D36" s="36">
+      <c r="D36" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E36" s="37">
+      <c r="E36" s="32">
         <v>0.157</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="35" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="36">
+      <c r="B37" s="31">
         <v>12332.2</v>
       </c>
-      <c r="C37" s="37">
+      <c r="C37" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D37" s="36">
+      <c r="D37" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E37" s="37">
+      <c r="E37" s="32">
         <v>0.155</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="35" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B38" s="36">
+      <c r="B38" s="31">
         <v>12815.4</v>
       </c>
-      <c r="C38" s="37">
+      <c r="C38" s="32">
         <v>6.3E-2</v>
       </c>
-      <c r="D38" s="36">
+      <c r="D38" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E38" s="37">
+      <c r="E38" s="32">
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="35" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B39" s="36">
+      <c r="B39" s="31">
         <v>13515.9</v>
       </c>
-      <c r="C39" s="37">
+      <c r="C39" s="32">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D39" s="36">
+      <c r="D39" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E39" s="37">
+      <c r="E39" s="32">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="35" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B40" s="36">
+      <c r="B40" s="31">
         <v>13768.3</v>
       </c>
-      <c r="C40" s="37">
+      <c r="C40" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D40" s="36">
+      <c r="D40" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E40" s="37">
+      <c r="E40" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="35" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B41" s="36">
+      <c r="B41" s="31">
         <v>14197.9</v>
       </c>
-      <c r="C41" s="37">
+      <c r="C41" s="32">
         <v>6.3E-2</v>
       </c>
-      <c r="D41" s="36">
+      <c r="D41" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E41" s="37">
+      <c r="E41" s="32">
         <v>0.08</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="34" t="s">
         <v>175</v>
       </c>
@@ -9765,218 +9765,218 @@
       <c r="D42" s="34"/>
       <c r="E42" s="34"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="35" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="36">
+      <c r="B43" s="31">
         <v>15989.6</v>
       </c>
-      <c r="C43" s="37">
+      <c r="C43" s="32">
         <v>6.2E-2</v>
       </c>
-      <c r="D43" s="36">
+      <c r="D43" s="31">
         <v>23118.6</v>
       </c>
-      <c r="E43" s="37">
+      <c r="E43" s="32">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="35" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="36">
+      <c r="B44" s="31">
         <v>16276.4</v>
       </c>
-      <c r="C44" s="37">
+      <c r="C44" s="32">
         <v>7.2999999999999995E-2</v>
       </c>
-      <c r="D44" s="36">
+      <c r="D44" s="31">
         <v>23118.6</v>
       </c>
-      <c r="E44" s="37">
+      <c r="E44" s="32">
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="35" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B45" s="36">
+      <c r="B45" s="31">
         <v>16312.3</v>
       </c>
-      <c r="C45" s="37">
+      <c r="C45" s="32">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="D45" s="36">
+      <c r="D45" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E45" s="37">
+      <c r="E45" s="32">
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="35" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="36">
+      <c r="B46" s="31">
         <v>17352.7</v>
       </c>
-      <c r="C46" s="37">
+      <c r="C46" s="32">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="D46" s="36">
+      <c r="D46" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E46" s="37">
+      <c r="E46" s="32">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="35" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="36">
+      <c r="B47" s="31">
         <v>18040.599999999999</v>
       </c>
-      <c r="C47" s="37">
+      <c r="C47" s="32">
         <v>0.08</v>
       </c>
-      <c r="D47" s="36">
+      <c r="D47" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E47" s="37">
+      <c r="E47" s="32">
         <v>0.125</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="35" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B48" s="36">
+      <c r="B48" s="31">
         <v>19187.2</v>
       </c>
-      <c r="C48" s="37">
+      <c r="C48" s="32">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="D48" s="36">
+      <c r="D48" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E48" s="37">
+      <c r="E48" s="32">
         <v>0.156</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="35" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B49" s="36">
+      <c r="B49" s="31">
         <v>20434.900000000001</v>
       </c>
-      <c r="C49" s="37">
+      <c r="C49" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D49" s="36">
+      <c r="D49" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E49" s="37">
+      <c r="E49" s="32">
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="35" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B50" s="36">
+      <c r="B50" s="31">
         <v>21174.1</v>
       </c>
-      <c r="C50" s="37">
+      <c r="C50" s="32">
         <v>0.09</v>
       </c>
-      <c r="D50" s="36">
+      <c r="D50" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E50" s="37">
+      <c r="E50" s="32">
         <v>0.16300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="35" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B51" s="36">
+      <c r="B51" s="31">
         <v>22411.1</v>
       </c>
-      <c r="C51" s="37">
+      <c r="C51" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D51" s="36">
+      <c r="D51" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E51" s="37">
+      <c r="E51" s="32">
         <v>0.13</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="35" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B52" s="36">
+      <c r="B52" s="31">
         <v>23219.599999999999</v>
       </c>
-      <c r="C52" s="37">
+      <c r="C52" s="32">
         <v>0.09</v>
       </c>
-      <c r="D52" s="36">
+      <c r="D52" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E52" s="37">
+      <c r="E52" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="35" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B53" s="36">
+      <c r="B53" s="31">
         <v>23981.5</v>
       </c>
-      <c r="C53" s="37">
+      <c r="C53" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D53" s="36">
+      <c r="D53" s="31">
         <v>23156.6</v>
       </c>
-      <c r="E53" s="37">
+      <c r="E53" s="32">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="35" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B54" s="36">
+      <c r="B54" s="31">
         <v>24826.7</v>
       </c>
-      <c r="C54" s="37">
+      <c r="C54" s="32">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="D54" s="36">
+      <c r="D54" s="31">
         <v>23156.6</v>
       </c>
-      <c r="E54" s="37">
+      <c r="E54" s="32">
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="38" t="s">
+    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="B55" s="38"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="38"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="35"/>
+      <c r="D55" s="35"/>
+      <c r="E55" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -9999,13 +9999,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" customWidth="1"/>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>119</v>
       </c>
@@ -10013,16 +10013,16 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>122</v>
       </c>
       <c r="B2">
-        <f>'Table 4.08'!B14</f>
-        <v>11225.7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <f>'Table 4.08'!B54</f>
+        <v>24826.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
     </row>
   </sheetData>
@@ -10037,12 +10037,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>146</v>
       </c>
@@ -10050,7 +10050,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>147</v>
       </c>

</xml_diff>

<commit_message>
Revert "Updated start year capacities to use the latest 860 with data for 2024 for plant and battery capacity"
This reverts commit 572a2dd1901f59815f85ceeb21ea968d5a5d5f2b.
</commit_message>
<xml_diff>
--- a/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
+++ b/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\GBSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\GBSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F54FC92-3C53-4C4D-9D96-341C82DD405A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68C85CB-F764-4BED-BCAC-5B594C512666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1268,8 +1268,20 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1277,6 +1289,9 @@
     </xf>
     <xf numFmtId="167" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1287,23 +1302,8 @@
     <xf numFmtId="167" fontId="22" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="74">
@@ -1683,23 +1683,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="60.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" customWidth="1"/>
+    <col min="2" max="2" width="60.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1707,84 +1707,84 @@
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="25" t="s">
         <v>149</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>1000</v>
       </c>
@@ -1801,14 +1801,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AK114"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.140625" customWidth="1"/>
-    <col min="2" max="2" width="45.7109375" customWidth="1"/>
+    <col min="1" max="1" width="32.08984375" customWidth="1"/>
+    <col min="2" max="2" width="45.7265625" customWidth="1"/>
     <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B1" s="9" t="s">
         <v>123</v>
       </c>
@@ -1915,8 +1915,8 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1927,7 +1927,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1951,7 +1951,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
@@ -1962,7 +1962,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1970,12 +1970,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="9" t="s">
         <v>9</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="10" t="s">
         <v>10</v>
       </c>
@@ -2195,18 +2195,18 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>13</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>-1.4527999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>-1.2109E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>2.2502999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>19</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>8.456E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>-5.6340000000000001E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="18" t="s">
         <v>25</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>0.123014</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>27</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>5.8900000000000003E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>2.3185000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
         <v>31</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
         <v>34</v>
       </c>
@@ -3449,12 +3449,12 @@
         <v>1.1344E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
         <v>37</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>-3.3660000000000001E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
         <v>39</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
         <v>41</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>-9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
         <v>42</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>-9.68E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>43</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>6.6000000000000005E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>44</v>
       </c>
@@ -4132,12 +4132,12 @@
         <v>-4.06E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>46</v>
       </c>
@@ -4250,7 +4250,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>47</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>48</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>49</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>50</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>52</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>53</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>54</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
         <v>55</v>
       </c>
@@ -5154,7 +5154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
         <v>56</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
         <v>58</v>
       </c>
@@ -5380,12 +5380,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
         <v>60</v>
       </c>
@@ -5498,7 +5498,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
         <v>61</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
         <v>62</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
         <v>63</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
         <v>64</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
         <v>65</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
         <v>66</v>
       </c>
@@ -6176,7 +6176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
         <v>67</v>
       </c>
@@ -6289,7 +6289,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
         <v>68</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
         <v>69</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>70</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
         <v>71</v>
       </c>
@@ -6741,12 +6741,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="12" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>73</v>
       </c>
@@ -6859,7 +6859,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
         <v>74</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="6" t="s">
         <v>75</v>
       </c>
@@ -7085,7 +7085,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
         <v>76</v>
       </c>
@@ -7198,7 +7198,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
         <v>77</v>
       </c>
@@ -7311,7 +7311,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
         <v>78</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="6" t="s">
         <v>79</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
         <v>80</v>
       </c>
@@ -7650,7 +7650,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="6" t="s">
         <v>81</v>
       </c>
@@ -7763,7 +7763,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
         <v>82</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
         <v>83</v>
       </c>
@@ -7989,12 +7989,12 @@
         <v>1.1053E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="6" t="s">
         <v>86</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>-9.3640000000000008E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
         <v>87</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>-2.039E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
         <v>89</v>
       </c>
@@ -8333,7 +8333,7 @@
         <v>2.5253000000000001E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
         <v>91</v>
       </c>
@@ -8446,7 +8446,7 @@
         <v>-7.0799999999999997E-4</v>
       </c>
     </row>
-    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
         <v>93</v>
       </c>
@@ -8559,7 +8559,7 @@
         <v>6.0502E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
         <v>94</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>4.0169999999999997E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="6" t="s">
         <v>96</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>4.7788999999999998E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="6" t="s">
         <v>97</v>
       </c>
@@ -8898,178 +8898,178 @@
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="33" t="s">
+    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B87" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C87" s="33"/>
-      <c r="D87" s="33"/>
-      <c r="E87" s="33"/>
-      <c r="F87" s="33"/>
-      <c r="G87" s="33"/>
-      <c r="H87" s="33"/>
-      <c r="I87" s="33"/>
-      <c r="J87" s="33"/>
-      <c r="K87" s="33"/>
-      <c r="L87" s="33"/>
-      <c r="M87" s="33"/>
-      <c r="N87" s="33"/>
-      <c r="O87" s="33"/>
-      <c r="P87" s="33"/>
-      <c r="Q87" s="33"/>
-      <c r="R87" s="33"/>
-      <c r="S87" s="33"/>
-      <c r="T87" s="33"/>
-      <c r="U87" s="33"/>
-      <c r="V87" s="33"/>
-      <c r="W87" s="33"/>
-      <c r="X87" s="33"/>
-      <c r="Y87" s="33"/>
-      <c r="Z87" s="33"/>
-      <c r="AA87" s="33"/>
-      <c r="AB87" s="33"/>
-      <c r="AC87" s="33"/>
-      <c r="AD87" s="33"/>
-      <c r="AE87" s="33"/>
-      <c r="AF87" s="33"/>
-      <c r="AG87" s="33"/>
-      <c r="AH87" s="33"/>
-      <c r="AI87" s="33"/>
-      <c r="AJ87" s="33"/>
-      <c r="AK87" s="33"/>
-    </row>
-    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C87" s="26"/>
+      <c r="D87" s="26"/>
+      <c r="E87" s="26"/>
+      <c r="F87" s="26"/>
+      <c r="G87" s="26"/>
+      <c r="H87" s="26"/>
+      <c r="I87" s="26"/>
+      <c r="J87" s="26"/>
+      <c r="K87" s="26"/>
+      <c r="L87" s="26"/>
+      <c r="M87" s="26"/>
+      <c r="N87" s="26"/>
+      <c r="O87" s="26"/>
+      <c r="P87" s="26"/>
+      <c r="Q87" s="26"/>
+      <c r="R87" s="26"/>
+      <c r="S87" s="26"/>
+      <c r="T87" s="26"/>
+      <c r="U87" s="26"/>
+      <c r="V87" s="26"/>
+      <c r="W87" s="26"/>
+      <c r="X87" s="26"/>
+      <c r="Y87" s="26"/>
+      <c r="Z87" s="26"/>
+      <c r="AA87" s="26"/>
+      <c r="AB87" s="26"/>
+      <c r="AC87" s="26"/>
+      <c r="AD87" s="26"/>
+      <c r="AE87" s="26"/>
+      <c r="AF87" s="26"/>
+      <c r="AG87" s="26"/>
+      <c r="AH87" s="26"/>
+      <c r="AI87" s="26"/>
+      <c r="AJ87" s="26"/>
+      <c r="AK87" s="26"/>
+    </row>
+    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B93" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B94" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B95" s="7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B96" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B97" s="7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B99" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B100" s="7" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B101" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B102" s="7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B103" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B104" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B105" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B106" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B107" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B108" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B109" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B110" s="7" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B111" s="7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B112" s="7" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B113" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B114" s="7" t="s">
         <v>138</v>
       </c>
@@ -9085,56 +9085,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46C8A405-A765-4E2E-A98F-140D5DD3A510}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.140625" style="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="26" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="26"/>
+    <col min="1" max="1" width="17.1796875" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="28"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="37" t="s">
+      <c r="C2" s="31"/>
+      <c r="D2" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="38"/>
-    </row>
-    <row r="3" spans="1:5" ht="51.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="E2" s="31"/>
+    </row>
+    <row r="3" spans="1:5" ht="26.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="33" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="34" t="s">
         <v>160</v>
       </c>
@@ -9143,194 +9143,194 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="30">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="35">
         <v>2014</v>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="36">
         <v>155.1</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="37">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="D5" s="31">
+      <c r="D5" s="36">
         <v>22477.9</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="37">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="30">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="35">
         <v>2015</v>
       </c>
-      <c r="B6" s="31">
+      <c r="B6" s="36">
         <v>206.8</v>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="37">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="36">
         <v>22568.9</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="37">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="30">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="35">
         <v>2016</v>
       </c>
-      <c r="B7" s="31">
+      <c r="B7" s="36">
         <v>423</v>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="37">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="36">
         <v>22752.7</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="37">
         <v>0.112</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="30">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="35">
         <v>2017</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="36">
         <v>632.79999999999995</v>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="37">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="36">
         <v>22791.7</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="37">
         <v>0.114</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="30">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="35">
         <v>2018</v>
       </c>
-      <c r="B9" s="31">
+      <c r="B9" s="36">
         <v>713.6</v>
       </c>
-      <c r="C9" s="32">
+      <c r="C9" s="37">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="36">
         <v>22815.4</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="37">
         <v>0.108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="30">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="35">
         <v>2019</v>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="36">
         <v>949.8</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="37">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="36">
         <v>22754.7</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="37">
         <v>0.104</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="30">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="35">
         <v>2020</v>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="36">
         <v>1210.3</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="37">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D11" s="31">
+      <c r="D11" s="36">
         <v>22939.599999999999</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="37">
         <v>0.105</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="30">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="35">
         <v>2021</v>
       </c>
-      <c r="B12" s="31">
+      <c r="B12" s="36">
         <v>2627.6</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="37">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="36">
         <v>23007.7</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="37">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="30">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="35">
         <v>2022</v>
       </c>
-      <c r="B13" s="31">
+      <c r="B13" s="36">
         <v>6566.1</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="37">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D13" s="31">
+      <c r="D13" s="36">
         <v>23033.9</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="37">
         <v>0.111</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="30">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="35">
         <v>2023</v>
       </c>
-      <c r="B14" s="31">
+      <c r="B14" s="36">
         <v>11225.7</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="37">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D14" s="31">
+      <c r="D14" s="36">
         <v>23132.1</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="37">
         <v>0.109</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="30">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="35">
         <v>2024</v>
       </c>
-      <c r="B15" s="31">
+      <c r="B15" s="36">
         <v>19945.099999999999</v>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="37">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D15" s="31">
+      <c r="D15" s="36">
         <v>23178.5</v>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="37">
         <v>0.114</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="34" t="s">
         <v>161</v>
       </c>
@@ -9339,211 +9339,211 @@
       <c r="D16" s="34"/>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="36">
         <v>4926.3999999999996</v>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="37">
         <v>5.5E-2</v>
       </c>
-      <c r="D17" s="31">
+      <c r="D17" s="36">
         <v>23013.4</v>
       </c>
-      <c r="E17" s="32">
+      <c r="E17" s="37">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="31">
+      <c r="B18" s="36">
         <v>4996.7</v>
       </c>
-      <c r="C18" s="32">
+      <c r="C18" s="37">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D18" s="31">
+      <c r="D18" s="36">
         <v>23013.4</v>
       </c>
-      <c r="E18" s="32">
+      <c r="E18" s="37">
         <v>8.8999999999999996E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="B19" s="31">
+      <c r="B19" s="36">
         <v>5069.2</v>
       </c>
-      <c r="C19" s="32">
+      <c r="C19" s="37">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="D19" s="31">
+      <c r="D19" s="36">
         <v>23013.4</v>
       </c>
-      <c r="E19" s="32">
+      <c r="E19" s="37">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="31">
+      <c r="B20" s="36">
         <v>5316.2</v>
       </c>
-      <c r="C20" s="32">
+      <c r="C20" s="37">
         <v>0.06</v>
       </c>
-      <c r="D20" s="31">
+      <c r="D20" s="36">
         <v>23013.4</v>
       </c>
-      <c r="E20" s="32">
+      <c r="E20" s="37">
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="35" t="s">
         <v>166</v>
       </c>
-      <c r="B21" s="31">
+      <c r="B21" s="36">
         <v>6055.5</v>
       </c>
-      <c r="C21" s="32">
+      <c r="C21" s="37">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D21" s="31">
+      <c r="D21" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E21" s="32">
+      <c r="E21" s="37">
         <v>0.109</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="31">
+      <c r="B22" s="36">
         <v>6064.5</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="37">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="D22" s="31">
+      <c r="D22" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E22" s="32">
+      <c r="E22" s="37">
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="31">
+      <c r="B23" s="36">
         <v>6555.2</v>
       </c>
-      <c r="C23" s="32">
+      <c r="C23" s="37">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D23" s="31">
+      <c r="D23" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="37">
         <v>0.159</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="B24" s="31">
+      <c r="B24" s="36">
         <v>6941.6</v>
       </c>
-      <c r="C24" s="32">
+      <c r="C24" s="37">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D24" s="31">
+      <c r="D24" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E24" s="32">
+      <c r="E24" s="37">
         <v>0.16400000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="36">
         <v>7469.9</v>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="37">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D25" s="31">
+      <c r="D25" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E25" s="32">
+      <c r="E25" s="37">
         <v>0.13200000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="B26" s="31">
+      <c r="B26" s="36">
         <v>7958.4</v>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="37">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E26" s="32">
+      <c r="E26" s="37">
         <v>8.4000000000000005E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="30" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="B27" s="31">
+      <c r="B27" s="36">
         <v>8630.7000000000007</v>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="37">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E27" s="32">
+      <c r="E27" s="37">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="36">
         <v>8696.4</v>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="37">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D28" s="31">
+      <c r="D28" s="36">
         <v>23043.9</v>
       </c>
-      <c r="E28" s="32">
+      <c r="E28" s="37">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="34" t="s">
         <v>174</v>
       </c>
@@ -9552,211 +9552,211 @@
       <c r="D29" s="34"/>
       <c r="E29" s="34"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="30" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="B30" s="31">
+      <c r="B30" s="36">
         <v>9168.7000000000007</v>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="37">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D30" s="31">
+      <c r="D30" s="36">
         <v>23057.8</v>
       </c>
-      <c r="E30" s="32">
+      <c r="E30" s="37">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="30" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="36">
         <v>9236.4</v>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="37">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="36">
         <v>23057.8</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="37">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="30" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="36">
         <v>9318.4</v>
       </c>
-      <c r="C32" s="32">
+      <c r="C32" s="37">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="36">
         <v>23137.8</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="37">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="30" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="B33" s="31">
+      <c r="B33" s="36">
         <v>9621.5</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="37">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="37">
         <v>8.7999999999999995E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="30" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="35" t="s">
         <v>166</v>
       </c>
-      <c r="B34" s="31">
+      <c r="B34" s="36">
         <v>9791.5</v>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="37">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D34" s="31">
+      <c r="D34" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="37">
         <v>0.109</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="30" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="B35" s="31">
+      <c r="B35" s="36">
         <v>9943.1</v>
       </c>
-      <c r="C35" s="32">
+      <c r="C35" s="37">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D35" s="31">
+      <c r="D35" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="37">
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="30" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="B36" s="31">
+      <c r="B36" s="36">
         <v>10846.6</v>
       </c>
-      <c r="C36" s="32">
+      <c r="C36" s="37">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D36" s="31">
+      <c r="D36" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="37">
         <v>0.157</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="30" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="31">
+      <c r="B37" s="36">
         <v>12332.2</v>
       </c>
-      <c r="C37" s="32">
+      <c r="C37" s="37">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D37" s="31">
+      <c r="D37" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E37" s="32">
+      <c r="E37" s="37">
         <v>0.155</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="30" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="B38" s="31">
+      <c r="B38" s="36">
         <v>12815.4</v>
       </c>
-      <c r="C38" s="32">
+      <c r="C38" s="37">
         <v>6.3E-2</v>
       </c>
-      <c r="D38" s="31">
+      <c r="D38" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E38" s="32">
+      <c r="E38" s="37">
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="30" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="B39" s="31">
+      <c r="B39" s="36">
         <v>13515.9</v>
       </c>
-      <c r="C39" s="32">
+      <c r="C39" s="37">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D39" s="31">
+      <c r="D39" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E39" s="32">
+      <c r="E39" s="37">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="30" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="B40" s="31">
+      <c r="B40" s="36">
         <v>13768.3</v>
       </c>
-      <c r="C40" s="32">
+      <c r="C40" s="37">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D40" s="31">
+      <c r="D40" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E40" s="32">
+      <c r="E40" s="37">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="30" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B41" s="31">
+      <c r="B41" s="36">
         <v>14197.9</v>
       </c>
-      <c r="C41" s="32">
+      <c r="C41" s="37">
         <v>6.3E-2</v>
       </c>
-      <c r="D41" s="31">
+      <c r="D41" s="36">
         <v>23147.4</v>
       </c>
-      <c r="E41" s="32">
+      <c r="E41" s="37">
         <v>0.08</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="34" t="s">
         <v>175</v>
       </c>
@@ -9765,218 +9765,218 @@
       <c r="D42" s="34"/>
       <c r="E42" s="34"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="30" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="31">
+      <c r="B43" s="36">
         <v>15989.6</v>
       </c>
-      <c r="C43" s="32">
+      <c r="C43" s="37">
         <v>6.2E-2</v>
       </c>
-      <c r="D43" s="31">
+      <c r="D43" s="36">
         <v>23118.6</v>
       </c>
-      <c r="E43" s="32">
+      <c r="E43" s="37">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="31">
+      <c r="B44" s="36">
         <v>16276.4</v>
       </c>
-      <c r="C44" s="32">
+      <c r="C44" s="37">
         <v>7.2999999999999995E-2</v>
       </c>
-      <c r="D44" s="31">
+      <c r="D44" s="36">
         <v>23118.6</v>
       </c>
-      <c r="E44" s="32">
+      <c r="E44" s="37">
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="30" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="B45" s="31">
+      <c r="B45" s="36">
         <v>16312.3</v>
       </c>
-      <c r="C45" s="32">
+      <c r="C45" s="37">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E45" s="32">
+      <c r="E45" s="37">
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="30" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="31">
+      <c r="B46" s="36">
         <v>17352.7</v>
       </c>
-      <c r="C46" s="32">
+      <c r="C46" s="37">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="D46" s="31">
+      <c r="D46" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E46" s="32">
+      <c r="E46" s="37">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="30" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="35" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="31">
+      <c r="B47" s="36">
         <v>18040.599999999999</v>
       </c>
-      <c r="C47" s="32">
+      <c r="C47" s="37">
         <v>0.08</v>
       </c>
-      <c r="D47" s="31">
+      <c r="D47" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E47" s="32">
+      <c r="E47" s="37">
         <v>0.125</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="30" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="B48" s="31">
+      <c r="B48" s="36">
         <v>19187.2</v>
       </c>
-      <c r="C48" s="32">
+      <c r="C48" s="37">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="D48" s="31">
+      <c r="D48" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E48" s="32">
+      <c r="E48" s="37">
         <v>0.156</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="30" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="35" t="s">
         <v>168</v>
       </c>
-      <c r="B49" s="31">
+      <c r="B49" s="36">
         <v>20434.900000000001</v>
       </c>
-      <c r="C49" s="32">
+      <c r="C49" s="37">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D49" s="31">
+      <c r="D49" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E49" s="32">
+      <c r="E49" s="37">
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="30" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="B50" s="31">
+      <c r="B50" s="36">
         <v>21174.1</v>
       </c>
-      <c r="C50" s="32">
+      <c r="C50" s="37">
         <v>0.09</v>
       </c>
-      <c r="D50" s="31">
+      <c r="D50" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E50" s="32">
+      <c r="E50" s="37">
         <v>0.16300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="30" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="B51" s="31">
+      <c r="B51" s="36">
         <v>22411.1</v>
       </c>
-      <c r="C51" s="32">
+      <c r="C51" s="37">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D51" s="31">
+      <c r="D51" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E51" s="32">
+      <c r="E51" s="37">
         <v>0.13</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="30" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="B52" s="31">
+      <c r="B52" s="36">
         <v>23219.599999999999</v>
       </c>
-      <c r="C52" s="32">
+      <c r="C52" s="37">
         <v>0.09</v>
       </c>
-      <c r="D52" s="31">
+      <c r="D52" s="36">
         <v>23198.6</v>
       </c>
-      <c r="E52" s="32">
+      <c r="E52" s="37">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="30" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="B53" s="31">
+      <c r="B53" s="36">
         <v>23981.5</v>
       </c>
-      <c r="C53" s="32">
+      <c r="C53" s="37">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D53" s="31">
+      <c r="D53" s="36">
         <v>23156.6</v>
       </c>
-      <c r="E53" s="32">
+      <c r="E53" s="37">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="30" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="B54" s="31">
+      <c r="B54" s="36">
         <v>24826.7</v>
       </c>
-      <c r="C54" s="32">
+      <c r="C54" s="37">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="36">
         <v>23156.6</v>
       </c>
-      <c r="E54" s="32">
+      <c r="E54" s="37">
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="35" t="s">
+    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="B55" s="35"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="35"/>
+      <c r="B55" s="38"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -9999,13 +9999,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="11.36328125" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>119</v>
       </c>
@@ -10013,16 +10013,16 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>122</v>
       </c>
       <c r="B2">
-        <f>'Table 4.08'!B54</f>
-        <v>24826.7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <f>'Table 4.08'!B14</f>
+        <v>11225.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B3" s="4"/>
     </row>
   </sheetData>
@@ -10037,12 +10037,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="1" max="1" width="28.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>146</v>
       </c>
@@ -10050,7 +10050,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="20" t="s">
         <v>147</v>
       </c>

</xml_diff>

<commit_message>
update start year GBSC, CCAMC
</commit_message>
<xml_diff>
--- a/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
+++ b/InputData/elec/GBSC/Grid Battery Storage Capacities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\GBSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\elec\GBSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68C85CB-F764-4BED-BCAC-5B594C512666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE802D1-3A1C-435A-A4C0-0F7764170732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1268,20 +1268,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1289,9 +1277,6 @@
     </xf>
     <xf numFmtId="167" fontId="29" fillId="20" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1302,8 +1287,23 @@
     <xf numFmtId="167" fontId="22" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="56">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="74">
@@ -1683,23 +1683,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" customWidth="1"/>
-    <col min="2" max="2" width="60.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1707,84 +1707,84 @@
         <v>152</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
         <v>2025</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
         <v>149</v>
       </c>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>1000</v>
       </c>
@@ -1801,14 +1801,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AK114"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.08984375" customWidth="1"/>
-    <col min="2" max="2" width="45.7265625" customWidth="1"/>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" customWidth="1"/>
     <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="9" t="s">
         <v>123</v>
       </c>
@@ -1915,8 +1915,8 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1927,7 +1927,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1951,7 +1951,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
@@ -1962,7 +1962,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1970,12 +1970,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
         <v>9</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="10" t="s">
         <v>10</v>
       </c>
@@ -2195,18 +2195,18 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>13</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>-1.4527999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>-1.2109E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>2.2502999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>19</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>8.456E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>-5.6340000000000001E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:37" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>25</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>0.123014</v>
       </c>
     </row>
-    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>27</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>5.8900000000000003E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>2.3185000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>31</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>34</v>
       </c>
@@ -3449,12 +3449,12 @@
         <v>1.1344E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>37</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>-3.3660000000000001E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>39</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>41</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>-9.9999999999999995E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>42</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>-9.68E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>43</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>6.6000000000000005E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>44</v>
       </c>
@@ -4132,12 +4132,12 @@
         <v>-4.06E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>46</v>
       </c>
@@ -4250,7 +4250,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>47</v>
       </c>
@@ -4363,7 +4363,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>48</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>49</v>
       </c>
@@ -4589,7 +4589,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>50</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>52</v>
       </c>
@@ -4815,7 +4815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>53</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>54</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>55</v>
       </c>
@@ -5154,7 +5154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>56</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>58</v>
       </c>
@@ -5380,12 +5380,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>60</v>
       </c>
@@ -5498,7 +5498,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>61</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>62</v>
       </c>
@@ -5724,7 +5724,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>63</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>64</v>
       </c>
@@ -5950,7 +5950,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>65</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>66</v>
       </c>
@@ -6176,7 +6176,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>67</v>
       </c>
@@ -6289,7 +6289,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>68</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>69</v>
       </c>
@@ -6515,7 +6515,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>70</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>71</v>
       </c>
@@ -6741,12 +6741,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="12" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>73</v>
       </c>
@@ -6859,7 +6859,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>74</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>75</v>
       </c>
@@ -7085,7 +7085,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>76</v>
       </c>
@@ -7198,7 +7198,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>77</v>
       </c>
@@ -7311,7 +7311,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>78</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>79</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>80</v>
       </c>
@@ -7650,7 +7650,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>81</v>
       </c>
@@ -7763,7 +7763,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>82</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>83</v>
       </c>
@@ -7989,12 +7989,12 @@
         <v>1.1053E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>86</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>-9.3640000000000008E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>87</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>-2.039E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>89</v>
       </c>
@@ -8333,7 +8333,7 @@
         <v>2.5253000000000001E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>91</v>
       </c>
@@ -8446,7 +8446,7 @@
         <v>-7.0799999999999997E-4</v>
       </c>
     </row>
-    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>93</v>
       </c>
@@ -8559,7 +8559,7 @@
         <v>6.0502E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>94</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>4.0169999999999997E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>96</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>4.7788999999999998E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>97</v>
       </c>
@@ -8898,178 +8898,178 @@
         <v>33</v>
       </c>
     </row>
-    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B87" s="26" t="s">
+    <row r="86" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="87" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="C87" s="26"/>
-      <c r="D87" s="26"/>
-      <c r="E87" s="26"/>
-      <c r="F87" s="26"/>
-      <c r="G87" s="26"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="26"/>
-      <c r="J87" s="26"/>
-      <c r="K87" s="26"/>
-      <c r="L87" s="26"/>
-      <c r="M87" s="26"/>
-      <c r="N87" s="26"/>
-      <c r="O87" s="26"/>
-      <c r="P87" s="26"/>
-      <c r="Q87" s="26"/>
-      <c r="R87" s="26"/>
-      <c r="S87" s="26"/>
-      <c r="T87" s="26"/>
-      <c r="U87" s="26"/>
-      <c r="V87" s="26"/>
-      <c r="W87" s="26"/>
-      <c r="X87" s="26"/>
-      <c r="Y87" s="26"/>
-      <c r="Z87" s="26"/>
-      <c r="AA87" s="26"/>
-      <c r="AB87" s="26"/>
-      <c r="AC87" s="26"/>
-      <c r="AD87" s="26"/>
-      <c r="AE87" s="26"/>
-      <c r="AF87" s="26"/>
-      <c r="AG87" s="26"/>
-      <c r="AH87" s="26"/>
-      <c r="AI87" s="26"/>
-      <c r="AJ87" s="26"/>
-      <c r="AK87" s="26"/>
-    </row>
-    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C87" s="33"/>
+      <c r="D87" s="33"/>
+      <c r="E87" s="33"/>
+      <c r="F87" s="33"/>
+      <c r="G87" s="33"/>
+      <c r="H87" s="33"/>
+      <c r="I87" s="33"/>
+      <c r="J87" s="33"/>
+      <c r="K87" s="33"/>
+      <c r="L87" s="33"/>
+      <c r="M87" s="33"/>
+      <c r="N87" s="33"/>
+      <c r="O87" s="33"/>
+      <c r="P87" s="33"/>
+      <c r="Q87" s="33"/>
+      <c r="R87" s="33"/>
+      <c r="S87" s="33"/>
+      <c r="T87" s="33"/>
+      <c r="U87" s="33"/>
+      <c r="V87" s="33"/>
+      <c r="W87" s="33"/>
+      <c r="X87" s="33"/>
+      <c r="Y87" s="33"/>
+      <c r="Z87" s="33"/>
+      <c r="AA87" s="33"/>
+      <c r="AB87" s="33"/>
+      <c r="AC87" s="33"/>
+      <c r="AD87" s="33"/>
+      <c r="AE87" s="33"/>
+      <c r="AF87" s="33"/>
+      <c r="AG87" s="33"/>
+      <c r="AH87" s="33"/>
+      <c r="AI87" s="33"/>
+      <c r="AJ87" s="33"/>
+      <c r="AK87" s="33"/>
+    </row>
+    <row r="88" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="7" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="7" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="7" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="7" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B106" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="7" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="7" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="7" t="s">
         <v>138</v>
       </c>
@@ -9085,56 +9085,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46C8A405-A765-4E2E-A98F-140D5DD3A510}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" style="28" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.1796875" style="28"/>
+    <col min="1" max="1" width="17.140625" style="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="26" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="31"/>
-    </row>
-    <row r="3" spans="1:5" ht="26.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="29" t="s">
+      <c r="E2" s="38"/>
+    </row>
+    <row r="3" spans="1:5" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="29" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
         <v>160</v>
       </c>
@@ -9143,194 +9143,194 @@
       <c r="D4" s="34"/>
       <c r="E4" s="34"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="30">
         <v>2014</v>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="31">
         <v>155.1</v>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="32">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="D5" s="36">
+      <c r="D5" s="31">
         <v>22477.9</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="30">
         <v>2015</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="31">
         <v>206.8</v>
       </c>
-      <c r="C6" s="37">
+      <c r="C6" s="32">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="D6" s="36">
+      <c r="D6" s="31">
         <v>22568.9</v>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="30">
         <v>2016</v>
       </c>
-      <c r="B7" s="36">
+      <c r="B7" s="31">
         <v>423</v>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="32">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="31">
         <v>22752.7</v>
       </c>
-      <c r="E7" s="37">
+      <c r="E7" s="32">
         <v>0.112</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="30">
         <v>2017</v>
       </c>
-      <c r="B8" s="36">
+      <c r="B8" s="31">
         <v>632.79999999999995</v>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="32">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="D8" s="36">
+      <c r="D8" s="31">
         <v>22791.7</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="32">
         <v>0.114</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="30">
         <v>2018</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B9" s="31">
         <v>713.6</v>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="32">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="31">
         <v>22815.4</v>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="32">
         <v>0.108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="30">
         <v>2019</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="31">
         <v>949.8</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="32">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="31">
         <v>22754.7</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="32">
         <v>0.104</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="30">
         <v>2020</v>
       </c>
-      <c r="B11" s="36">
+      <c r="B11" s="31">
         <v>1210.3</v>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="32">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="31">
         <v>22939.599999999999</v>
       </c>
-      <c r="E11" s="37">
+      <c r="E11" s="32">
         <v>0.105</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="30">
         <v>2021</v>
       </c>
-      <c r="B12" s="36">
+      <c r="B12" s="31">
         <v>2627.6</v>
       </c>
-      <c r="C12" s="37">
+      <c r="C12" s="32">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="31">
         <v>23007.7</v>
       </c>
-      <c r="E12" s="37">
+      <c r="E12" s="32">
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="30">
         <v>2022</v>
       </c>
-      <c r="B13" s="36">
+      <c r="B13" s="31">
         <v>6566.1</v>
       </c>
-      <c r="C13" s="37">
+      <c r="C13" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="31">
         <v>23033.9</v>
       </c>
-      <c r="E13" s="37">
+      <c r="E13" s="32">
         <v>0.111</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="30">
         <v>2023</v>
       </c>
-      <c r="B14" s="36">
+      <c r="B14" s="31">
         <v>11225.7</v>
       </c>
-      <c r="C14" s="37">
+      <c r="C14" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="31">
         <v>23132.1</v>
       </c>
-      <c r="E14" s="37">
+      <c r="E14" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="30">
         <v>2024</v>
       </c>
-      <c r="B15" s="36">
+      <c r="B15" s="31">
         <v>19945.099999999999</v>
       </c>
-      <c r="C15" s="37">
+      <c r="C15" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="31">
         <v>23178.5</v>
       </c>
-      <c r="E15" s="37">
+      <c r="E15" s="32">
         <v>0.114</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
         <v>161</v>
       </c>
@@ -9339,211 +9339,211 @@
       <c r="D16" s="34"/>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="35" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="36">
+      <c r="B17" s="31">
         <v>4926.3999999999996</v>
       </c>
-      <c r="C17" s="37">
+      <c r="C17" s="32">
         <v>5.5E-2</v>
       </c>
-      <c r="D17" s="36">
+      <c r="D17" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E17" s="37">
+      <c r="E17" s="32">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="35" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="36">
+      <c r="B18" s="31">
         <v>4996.7</v>
       </c>
-      <c r="C18" s="37">
+      <c r="C18" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="32">
         <v>8.8999999999999996E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="35" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B19" s="36">
+      <c r="B19" s="31">
         <v>5069.2</v>
       </c>
-      <c r="C19" s="37">
+      <c r="C19" s="32">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="D19" s="36">
+      <c r="D19" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E19" s="37">
+      <c r="E19" s="32">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="35" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="36">
+      <c r="B20" s="31">
         <v>5316.2</v>
       </c>
-      <c r="C20" s="37">
+      <c r="C20" s="32">
         <v>0.06</v>
       </c>
-      <c r="D20" s="36">
+      <c r="D20" s="31">
         <v>23013.4</v>
       </c>
-      <c r="E20" s="37">
+      <c r="E20" s="32">
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="35" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B21" s="36">
+      <c r="B21" s="31">
         <v>6055.5</v>
       </c>
-      <c r="C21" s="37">
+      <c r="C21" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D21" s="36">
+      <c r="D21" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E21" s="37">
+      <c r="E21" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="35" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="31">
         <v>6064.5</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="32">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="D22" s="36">
+      <c r="D22" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E22" s="37">
+      <c r="E22" s="32">
         <v>0.14799999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="35" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B23" s="36">
+      <c r="B23" s="31">
         <v>6555.2</v>
       </c>
-      <c r="C23" s="37">
+      <c r="C23" s="32">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E23" s="37">
+      <c r="E23" s="32">
         <v>0.159</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="35" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B24" s="36">
+      <c r="B24" s="31">
         <v>6941.6</v>
       </c>
-      <c r="C24" s="37">
+      <c r="C24" s="32">
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="D24" s="36">
+      <c r="D24" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E24" s="37">
+      <c r="E24" s="32">
         <v>0.16400000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="35" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B25" s="36">
+      <c r="B25" s="31">
         <v>7469.9</v>
       </c>
-      <c r="C25" s="37">
+      <c r="C25" s="32">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="D25" s="36">
+      <c r="D25" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E25" s="37">
+      <c r="E25" s="32">
         <v>0.13200000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="35" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B26" s="36">
+      <c r="B26" s="31">
         <v>7958.4</v>
       </c>
-      <c r="C26" s="37">
+      <c r="C26" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D26" s="36">
+      <c r="D26" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E26" s="37">
+      <c r="E26" s="32">
         <v>8.4000000000000005E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="35" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B27" s="36">
+      <c r="B27" s="31">
         <v>8630.7000000000007</v>
       </c>
-      <c r="C27" s="37">
+      <c r="C27" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D27" s="36">
+      <c r="D27" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E27" s="37">
+      <c r="E27" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="35" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="31">
         <v>8696.4</v>
       </c>
-      <c r="C28" s="37">
+      <c r="C28" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="31">
         <v>23043.9</v>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="32">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="34" t="s">
         <v>174</v>
       </c>
@@ -9552,211 +9552,211 @@
       <c r="D29" s="34"/>
       <c r="E29" s="34"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="35" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="31">
         <v>9168.7000000000007</v>
       </c>
-      <c r="C30" s="37">
+      <c r="C30" s="32">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="D30" s="36">
+      <c r="D30" s="31">
         <v>23057.8</v>
       </c>
-      <c r="E30" s="37">
+      <c r="E30" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="35" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B31" s="36">
+      <c r="B31" s="31">
         <v>9236.4</v>
       </c>
-      <c r="C31" s="37">
+      <c r="C31" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D31" s="36">
+      <c r="D31" s="31">
         <v>23057.8</v>
       </c>
-      <c r="E31" s="37">
+      <c r="E31" s="32">
         <v>9.6000000000000002E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="35" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B32" s="36">
+      <c r="B32" s="31">
         <v>9318.4</v>
       </c>
-      <c r="C32" s="37">
+      <c r="C32" s="32">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D32" s="36">
+      <c r="D32" s="31">
         <v>23137.8</v>
       </c>
-      <c r="E32" s="37">
+      <c r="E32" s="32">
         <v>9.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="35" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="31">
         <v>9621.5</v>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="32">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E33" s="37">
+      <c r="E33" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="35" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B34" s="36">
+      <c r="B34" s="31">
         <v>9791.5</v>
       </c>
-      <c r="C34" s="37">
+      <c r="C34" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D34" s="36">
+      <c r="D34" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E34" s="37">
+      <c r="E34" s="32">
         <v>0.109</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="35" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B35" s="36">
+      <c r="B35" s="31">
         <v>9943.1</v>
       </c>
-      <c r="C35" s="37">
+      <c r="C35" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D35" s="36">
+      <c r="D35" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E35" s="37">
+      <c r="E35" s="32">
         <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="35" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="31">
         <v>10846.6</v>
       </c>
-      <c r="C36" s="37">
+      <c r="C36" s="32">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="D36" s="36">
+      <c r="D36" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E36" s="37">
+      <c r="E36" s="32">
         <v>0.157</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="35" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B37" s="36">
+      <c r="B37" s="31">
         <v>12332.2</v>
       </c>
-      <c r="C37" s="37">
+      <c r="C37" s="32">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D37" s="36">
+      <c r="D37" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E37" s="37">
+      <c r="E37" s="32">
         <v>0.155</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="35" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B38" s="36">
+      <c r="B38" s="31">
         <v>12815.4</v>
       </c>
-      <c r="C38" s="37">
+      <c r="C38" s="32">
         <v>6.3E-2</v>
       </c>
-      <c r="D38" s="36">
+      <c r="D38" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E38" s="37">
+      <c r="E38" s="32">
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="35" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B39" s="36">
+      <c r="B39" s="31">
         <v>13515.9</v>
       </c>
-      <c r="C39" s="37">
+      <c r="C39" s="32">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D39" s="36">
+      <c r="D39" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E39" s="37">
+      <c r="E39" s="32">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="35" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B40" s="36">
+      <c r="B40" s="31">
         <v>13768.3</v>
       </c>
-      <c r="C40" s="37">
+      <c r="C40" s="32">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="D40" s="36">
+      <c r="D40" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E40" s="37">
+      <c r="E40" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="35" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B41" s="36">
+      <c r="B41" s="31">
         <v>14197.9</v>
       </c>
-      <c r="C41" s="37">
+      <c r="C41" s="32">
         <v>6.3E-2</v>
       </c>
-      <c r="D41" s="36">
+      <c r="D41" s="31">
         <v>23147.4</v>
       </c>
-      <c r="E41" s="37">
+      <c r="E41" s="32">
         <v>0.08</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="34" t="s">
         <v>175</v>
       </c>
@@ -9765,218 +9765,218 @@
       <c r="D42" s="34"/>
       <c r="E42" s="34"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="35" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="36">
+      <c r="B43" s="31">
         <v>15989.6</v>
       </c>
-      <c r="C43" s="37">
+      <c r="C43" s="32">
         <v>6.2E-2</v>
       </c>
-      <c r="D43" s="36">
+      <c r="D43" s="31">
         <v>23118.6</v>
       </c>
-      <c r="E43" s="37">
+      <c r="E43" s="32">
         <v>9.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="35" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="36">
+      <c r="B44" s="31">
         <v>16276.4</v>
       </c>
-      <c r="C44" s="37">
+      <c r="C44" s="32">
         <v>7.2999999999999995E-2</v>
       </c>
-      <c r="D44" s="36">
+      <c r="D44" s="31">
         <v>23118.6</v>
       </c>
-      <c r="E44" s="37">
+      <c r="E44" s="32">
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="35" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="B45" s="36">
+      <c r="B45" s="31">
         <v>16312.3</v>
       </c>
-      <c r="C45" s="37">
+      <c r="C45" s="32">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="D45" s="36">
+      <c r="D45" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E45" s="37">
+      <c r="E45" s="32">
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="35" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="30" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="36">
+      <c r="B46" s="31">
         <v>17352.7</v>
       </c>
-      <c r="C46" s="37">
+      <c r="C46" s="32">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="D46" s="36">
+      <c r="D46" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E46" s="37">
+      <c r="E46" s="32">
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="35" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="36">
+      <c r="B47" s="31">
         <v>18040.599999999999</v>
       </c>
-      <c r="C47" s="37">
+      <c r="C47" s="32">
         <v>0.08</v>
       </c>
-      <c r="D47" s="36">
+      <c r="D47" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E47" s="37">
+      <c r="E47" s="32">
         <v>0.125</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="35" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="B48" s="36">
+      <c r="B48" s="31">
         <v>19187.2</v>
       </c>
-      <c r="C48" s="37">
+      <c r="C48" s="32">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="D48" s="36">
+      <c r="D48" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E48" s="37">
+      <c r="E48" s="32">
         <v>0.156</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="35" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="B49" s="36">
+      <c r="B49" s="31">
         <v>20434.900000000001</v>
       </c>
-      <c r="C49" s="37">
+      <c r="C49" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D49" s="36">
+      <c r="D49" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E49" s="37">
+      <c r="E49" s="32">
         <v>0.16800000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="35" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="B50" s="36">
+      <c r="B50" s="31">
         <v>21174.1</v>
       </c>
-      <c r="C50" s="37">
+      <c r="C50" s="32">
         <v>0.09</v>
       </c>
-      <c r="D50" s="36">
+      <c r="D50" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E50" s="37">
+      <c r="E50" s="32">
         <v>0.16300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="35" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="B51" s="36">
+      <c r="B51" s="31">
         <v>22411.1</v>
       </c>
-      <c r="C51" s="37">
+      <c r="C51" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="D51" s="36">
+      <c r="D51" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E51" s="37">
+      <c r="E51" s="32">
         <v>0.13</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="35" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="30" t="s">
         <v>171</v>
       </c>
-      <c r="B52" s="36">
+      <c r="B52" s="31">
         <v>23219.599999999999</v>
       </c>
-      <c r="C52" s="37">
+      <c r="C52" s="32">
         <v>0.09</v>
       </c>
-      <c r="D52" s="36">
+      <c r="D52" s="31">
         <v>23198.6</v>
       </c>
-      <c r="E52" s="37">
+      <c r="E52" s="32">
         <v>8.3000000000000004E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="35" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="B53" s="36">
+      <c r="B53" s="31">
         <v>23981.5</v>
       </c>
-      <c r="C53" s="37">
+      <c r="C53" s="32">
         <v>8.7999999999999995E-2</v>
       </c>
-      <c r="D53" s="36">
+      <c r="D53" s="31">
         <v>23156.6</v>
       </c>
-      <c r="E53" s="37">
+      <c r="E53" s="32">
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="35" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="B54" s="36">
+      <c r="B54" s="31">
         <v>24826.7</v>
       </c>
-      <c r="C54" s="37">
+      <c r="C54" s="32">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="D54" s="36">
+      <c r="D54" s="31">
         <v>23156.6</v>
       </c>
-      <c r="E54" s="37">
+      <c r="E54" s="32">
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="38" t="s">
+    <row r="55" spans="1:5" ht="336" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="35" t="s">
         <v>176</v>
       </c>
-      <c r="B55" s="38"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="38"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="35"/>
+      <c r="D55" s="35"/>
+      <c r="E55" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -9999,13 +9999,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.36328125" customWidth="1"/>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>119</v>
       </c>
@@ -10013,16 +10013,16 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>122</v>
       </c>
       <c r="B2">
-        <f>'Table 4.08'!B14</f>
-        <v>11225.7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <f>'Table 4.08'!B15</f>
+        <v>19945.099999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="4"/>
     </row>
   </sheetData>
@@ -10037,12 +10037,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.08984375" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>146</v>
       </c>
@@ -10050,7 +10050,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>147</v>
       </c>

</xml_diff>